<commit_message>
feat: finish worksheet-specific deduction updates
</commit_message>
<xml_diff>
--- a/Data/RebateTemplates/andres-asw.xlsx
+++ b/Data/RebateTemplates/andres-asw.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="1" r:id="Ra077450a986e4c61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monto de factura" sheetId="2" r:id="R64ad21dca1164e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REBAJO" sheetId="3" r:id="Rb4d159ffda0447e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="1" r:id="R650e5abf83c74aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monto de factura" sheetId="2" r:id="Rb5c6371de7fc4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REBAJO" sheetId="3" r:id="R8e482edd44b248ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10047,7 +10047,7 @@
         <x:v>460</x:v>
       </x:c>
       <x:c r="G1" t="str">
-        <x:v>TC FIJO</x:v>
+        <x:v>TC</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>